<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.001-08 Le château de la rive
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.001-08.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.001-08.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorina veut un château sur la rive. Le seau goutte, elle l'essuie, hésite, le met dans le sac. Le mur de sable tient.</t>
+          <t>Sur la table du jardin, la poussière est tiède. Un éclat de caillou luit dans le dessin du château. Victorina veut le vrai château à la rive, maintenant. Elle pousse tout dans le sac : le zip mord, l'éclat roule sous le banc. Papa s'accroupit. Une chose, puis la suivante. Sur le sentier, elle pose le sac, part avec le seau. Elle refuse de foncer, reprend le sac. Dans le mur, l'éclat de caillou garde un bord humide.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le sable de la rive est encore froid. L'eau du fleuve cliquette contre les cailloux. Le robinet du jardin goutte encore. Une goutte tombe dans le seau rouge. Le plastique fait un petit toc. L'herbe est encore mouillée. Les bottes brillent un peu. L'entrée sent l'herbe coupée. Un arrosoir attend près des bottes. Le métal est un peu froid. Une abeille passe tout bas. Victorina, on va à la rive. Je veux un château de sable. Avec le seau, alors. En ce moment, Victorina touche le seau. Le plastique est un peu froid. Papa pose le sac près de la porte. Prends de l'eau, la rive est au soleil. Victorina met la gourde dans le sac. La gourde est fraîche. Une goutte glisse du seau. Elle tombe sur le tapis. Le seau est mouillé. On l'essuie, puis dans le sac. Victorina essuie le bord. Elle hésite. Le seau reste un moment dehors. Le château a besoin du seau. Il est encore un peu mouillé. Tu l'essuies encore ? Oui. Victorina passe le torchon une fois de plus. Le plastique n'est plus luisant.</t>
+          <t>Sur la table du jardin, la poussière est tiède. Victorina dessine un château, du doigt. Le doigt bute contre un éclat de caillou. Le petit morceau luit, pâle. Il brille, papa. C'est un morceau du chemin. Elle le pose au milieu du dessin. C'est ma fenêtre. Derrière la haie, le fleuve clapote. L'air sent l'herbe coupée et l'eau. Les bottes attendent près de l'arrosoir. Victorina, on va à la rive. Je veux mon château, maintenant ! Avec le seau, et le sac. Le seau rouge attend près des bottes. En ce moment, Victorina saisit le sac. Le tissu gratte sous ses doigts. Prends de l'eau, la rive est au soleil. Victorina prend la gourde froide. Le bouchon fait un petit clic. Je mets tout, d'un coup ! Elle pousse gourde, seau et pelle. Le zip mord le manche de la pelle. Le seau bascule, tape la dalle. L'éclat de caillou roule sous le banc. Ça reste coincé ! Le sourire de Victorina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le sable de la rive est encore froid. L'eau du fleuve cliquette contre les cailloux. Le robinet du jardin goutte encore. Une goutte tombe dans le seau rouge. Le plastique fait un petit toc. L'herbe est encore mouillée. Les bottes brillent un peu. L'entrée sent l'herbe coupée. Un arrosoir attend près des bottes. Le métal est un peu froid. Une abeille passe tout bas. Victorina, on va à la rive. Je veux un château de sable. Avec le seau, alors. En ce moment, Victorina touche le seau. Le plastique est un peu froid. Papa pose le sac près de la porte. Prends de l'eau, la rive est au soleil. Victorina met la gourde dans le sac. La gourde est fraîche. Une goutte glisse du seau. Elle tombe sur le tapis. Le seau est mouillé. On l'essuie, puis dans le sac. Victorina essuie le bord. Elle hésite. Le seau reste un moment dehors. Le château a besoin du seau. Il est encore un peu mouillé. Tu l'essuies encore ? Oui. Victorina passe le torchon une fois de plus. Le plastique n'est plus luisant.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sur la table du jardin, la poussière est tiède. Victorina dessine un château, du doigt. Le doigt bute contre un &lt;emphasis level="moderate"&gt;éclat de caillou&lt;/emphasis&gt;. Le petit morceau luit, pâle. Il brille, papa. C'est un morceau du chemin. Elle le pose au milieu du dessin. C'est ma fenêtre. Derrière la haie, le fleuve clapote. L'air sent l'herbe coupée et l'eau. Les bottes attendent près de l'arrosoir. Victorina, on va à la rive. Je veux mon château, maintenant ! Avec le seau, et le sac. Le seau rouge attend près des bottes. En ce moment, Victorina saisit le sac. Le tissu gratte sous ses doigts. Prends de l'eau, la rive est au soleil. Victorina prend la gourde froide. Le bouchon fait un petit clic. Je mets tout, d'un coup ! Elle pousse gourde, seau et pelle. Le zip mord le manche de la pelle. Le seau bascule, tape la dalle. L'éclat de caillou roule sous le banc. Ça reste coincé ! Le sourire de Victorina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Florence va au parc. Papa pose le &lt;emphasis&gt;sac&lt;/emphasis&gt; près de la porte. Papa dit : la gourde, le seau. Florence met la gourde dans le sac. Elle met le seau. Parce que l'adulte a dit ces choses, elle les met. Le sac est prêt. Maman vérifie. Florence dit : c'est ce que l'adulte a dit. Dans le sac. La gourde est fraîche. Le seau est rouge. Papa ouvre la porte. [pause]</t>
+          <t>Sur la table du jardin, la poussière est tiède. Victorina dessine un château, du doigt. Le doigt bute contre un &lt;emphasis&gt;éclat de caillou&lt;/emphasis&gt;. Le petit morceau luit, pâle. Il brille, papa. C'est un morceau du chemin. Elle le pose au milieu du dessin. C'est ma fenêtre. Derrière la haie, le fleuve clapote. L'air sent l'herbe coupée et l'eau. Les bottes attendent près de l'arrosoir. Victorina, on va à la rive. Je veux mon château, maintenant ! Avec le seau, et le sac. Le seau rouge attend près des bottes. En ce moment, Victorina saisit le sac. Le tissu gratte sous ses doigts. Prends de l'eau, la rive est au soleil. Victorina prend la gourde froide. Le bouchon fait un petit clic. Je mets tout, d'un coup ! Elle pousse gourde, seau et pelle. Le zip mord le manche de la pelle. Le seau bascule, tape la dalle. L'éclat de caillou roule sous le banc. Ça reste coincé ! Le sourire de Victorina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>éclat de caillou</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,47 +1321,46 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_chateau_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le sable de la rive est encore froid.
-narrateur|L'eau du fleuve cliquette contre les cailloux.
-narrateur|Le robinet du jardin goutte encore.
-narrateur|Une goutte tombe dans le seau rouge.
-narrateur|Le plastique fait un petit toc.
-narrateur|L'herbe est encore mouillée.
-narrateur|Les bottes brillent un peu.
-narrateur|L'entrée sent l'herbe coupée.
-narrateur|Un arrosoir attend près des bottes.
-narrateur|Le métal est un peu froid.
-narrateur|Une abeille passe tout bas.
+          <t>narrateur|Sur la table du jardin, la poussière est tiède.
+narrateur|Victorina dessine un château, du doigt.
+narrateur|Le doigt bute contre un éclat de caillou.
+narrateur|Le petit morceau luit, pâle.
+enfant-f|Il brille, papa.
+papa|C'est un morceau du chemin.
+narrateur|Elle le pose au milieu du dessin.
+enfant-f|C'est ma fenêtre.
+narrateur|Derrière la haie, le fleuve clapote.
+narrateur|L'air sent l'herbe coupée et l'eau.
+narrateur|Les bottes attendent près de l'arrosoir.
 maman|Victorina, on va à la rive.
-enfant-f|Je veux un château de sable.
-maman|Avec le seau, alors.
-narrateur|En ce moment, Victorina touche le seau.
-narrateur|Le plastique est un peu froid.
-narrateur|Papa pose le sac près de la porte.
+enfant-f|Je veux mon château, maintenant !
+maman|Avec le seau, et le sac.
+narrateur|Le seau rouge attend près des bottes.
+narrateur|En ce moment, Victorina saisit le sac.
+narrateur|Le tissu gratte sous ses doigts.
 papa|Prends de l'eau, la rive est au soleil.
-narrateur|Victorina met la gourde dans le sac.
-narrateur|La gourde est fraîche.
-narrateur|Une goutte glisse du seau.
-narrateur|Elle tombe sur le tapis.
-enfant-f|Le seau est mouillé.
-papa|On l'essuie, puis dans le sac.
-narrateur|Victorina essuie le bord.
-narrateur|Elle hésite.
-narrateur|Le seau reste un moment dehors.
-maman|Le château a besoin du seau.
-enfant-f|Il est encore un peu mouillé.
-papa|Tu l'essuies encore ?
-enfant-f|Oui.
-narrateur|Victorina passe le torchon une fois de plus.
-narrateur|Le plastique n'est plus luisant.</t>
+narrateur|Victorina prend la gourde froide.
+narrateur|Le bouchon fait un petit clic.
+enfant-f|Je mets tout, d'un coup !
+narrateur|Elle pousse gourde, seau et pelle.
+narrateur|Le zip mord le manche de la pelle.
+narrateur|Le seau bascule, tape la dalle.
+narrateur|L'éclat de caillou roule sous le banc.
+enfant-f|Ça reste coincé !
+narrateur|Le sourire de Victorina disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>jardin,dalle,arrosoir</t>
         </is>
       </c>
     </row>
@@ -1393,12 +1392,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorina prépare le sac. Où met-elle les affaires ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorina prépare le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. Où met-elle les affaires ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Florence prépare le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Que met-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Victorina prépare le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Où met-elle les affaires ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1461,7 +1460,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1472,7 +1471,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1487,11 +1486,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1502,23 +1501,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1533,17 +1532,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=les_affaires_vont_dans_le_sac; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1576,17 +1575,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Le seau vient avec nous. Victorina prend le seau rouge. Elle le met dans le sac. Merci, Victorina. Victorina ferme le sac. Ça fait zzz. Le sac est prêt. La gourde est dedans ? Oui, et le seau aussi. Le sac est prêt ? Oui, papa. Dans le sac, la gourde est fraîche. Le seau aussi. Pour le château. Oui, on l'emporte. On met tes bottes ? Oui.</t>
+          <t>Papa s'accroupit à la même hauteur. Sors la pelle, d'abord. Victorina tire le manche coincé. Le zip lâche, petit à petit. L'eau va au fond. Elle range la gourde froide. Le seau rouge glisse à côté. Et mon éclat ? L'éclat de caillou n'est pas sur la dalle. Regarde sous le banc ? Victorina se baisse près du bois. Ses doigts trouvent le bord lisse. Il était caché. Elle le glisse dans la poche du sac. Le zip avance, sans mordre. Merci, Victorina. Il part. Le sac est prêt ? Oui, papa. Tu prends aussi tes bottes ? Oui, pour le château. Victorina pose la main sur le tissu. Le tissu est un peu rêche.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Le seau vient avec nous. Victorina prend le seau rouge. Elle le met dans le sac. Merci, Victorina. Victorina ferme le sac. Ça fait zzz. Le sac est prêt. La gourde est dedans ? Oui, et le seau aussi. Le sac est prêt ? Oui, papa. Dans le sac, la gourde est fraîche. Le seau aussi. Pour le château. Oui, on l'emporte. On met tes bottes ? Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa s'accroupit à la même hauteur. Sors la pelle, d'abord. Victorina tire le manche coincé. Le zip lâche, petit à petit. L'eau va au fond. Elle range la gourde froide. Le seau rouge glisse à côté. Et mon éclat ? L'&lt;emphasis level="moderate"&gt;éclat de caillou&lt;/emphasis&gt; n'est pas sur la dalle. Regarde sous le banc ? Victorina se baisse près du bois. Ses doigts trouvent le bord lisse. Il était caché. Elle le glisse dans la poche du sac. Le zip avance, sans mordre. Merci, Victorina. Il part. Le sac est prêt ? Oui, papa. Tu prends aussi tes bottes ? Oui, pour le château. Victorina pose la main sur le tissu. Le tissu est un peu rêche.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Florence a préparé le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Elle a mis ce que l'adulte a dit. Papa et maman étaient là. [pause]</t>
+          <t>Papa s'accroupit à la même hauteur. Sors la pelle, d'abord. Victorina tire le manche coincé. Le zip lâche, petit à petit. L'eau va au fond. Elle range la gourde froide. Le seau rouge glisse à côté. Et mon éclat ? L'&lt;emphasis&gt;éclat de caillou&lt;/emphasis&gt; n'est pas sur la dalle. Regarde sous le banc ? Victorina se baisse près du bois. Ses doigts trouvent le bord lisse. Il était caché. Elle le glisse dans la poche du sac. Le zip avance, sans mordre. Merci, Victorina. Il part. Le sac est prêt ? Oui, papa. Tu prends aussi tes bottes ? Oui, pour le château. Victorina pose la main sur le tissu. Le tissu est un peu rêche. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1644,7 +1643,7 @@
         <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1667,7 +1666,7 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>éclat de caillou</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
@@ -1681,16 +1680,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1715,28 +1714,39 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=une_chose_puis_la_suivante; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>maman|Le seau vient avec nous.
-narrateur|Victorina prend le seau rouge.
-narrateur|Elle le met dans le sac.
+          <t>narrateur|Papa s'accroupit à la même hauteur.
+papa|Sors la pelle, d'abord.
+narrateur|Victorina tire le manche coincé.
+narrateur|Le zip lâche, petit à petit.
+maman|L'eau va au fond.
+narrateur|Elle range la gourde froide.
+narrateur|Le seau rouge glisse à côté.
+enfant-f|Et mon éclat ?
+narrateur|L'éclat de caillou n'est pas sur la dalle.
+papa|Regarde sous le banc ?
+narrateur|Victorina se baisse près du bois.
+narrateur|Ses doigts trouvent le bord lisse.
+enfant-f|Il était caché.
+narrateur|Elle le glisse dans la poche du sac.
+narrateur|Le zip avance, sans mordre.
 papa|Merci, Victorina.
-narrateur|Victorina ferme le sac.
-narrateur|Ça fait zzz.
-narrateur|Le sac est prêt.
-maman|La gourde est dedans ?
-enfant-f|Oui, et le seau aussi.
+enfant-f|Il part.
 papa|Le sac est prêt ?
 enfant-f|Oui, papa.
-narrateur|Dans le sac, la gourde est fraîche.
-maman|Le seau aussi.
-enfant-f|Pour le château.
-papa|Oui, on l'emporte.
-papa|On met tes bottes ?
-enfant-f|Oui.</t>
+maman|Tu prends aussi tes bottes ?
+enfant-f|Oui, pour le château.
+narrateur|Victorina pose la main sur le tissu.
+narrateur|Le tissu est un peu rêche.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>zip,sac</t>
         </is>
       </c>
     </row>
@@ -1763,17 +1773,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On met tes bottes. Victorina enfile ses bottes. Tu as fini tes bottes ? Oui, papa. On ferme la porte. Papa ferme la porte. Tu as ton sac, Victorina ? Oui, maman. Le chemin sent l'herbe mouillée, puis le fleuve. Le seau tape un peu, tout doux. Mon château va être grand. Oui, le sable t'attend. Ils arrivent à la rive. Le sable est encore un peu frais. Victorina pose le sac. Elle sort le seau. Le plastique n'est plus mouillé. Je fais le mur. Doucement, une poignée, puis une autre. Le sable fait un petit bruit. Un mur tout bas apparaît. Il tient, ce mur. Encore une poignée. Victorina appuie tout doucement. Le château a un petit coin rond.</t>
+          <t>On met tes bottes. Victorina enfile ses bottes. Tu as fini tes bottes ? Oui, papa. On ferme la porte. Papa ferme la porte. Tu as ton sac, Victorina ? Oui, maman. Le chemin sent l'herbe, puis le fleuve. Le seau tape un peu contre sa hanche. Mon château va être grand ! Oui, le sable t'attend. Le sable luisant appelle, au bout du sentier. J'y vais avec le seau ! Elle pose le sac contre une racine. Elle part avec le seau seul. La poche vide manque sur sa hanche. Mon éclat ! Victorina s'arrête net. Elle refuse de foncer. Attends, je regarde. Le sac attend contre la racine. Dans la poche, l'éclat de caillou pèse. Tu le sens, dans le sac ? Oui. Elle revient, prend le sac. La sangle revient sur l'épaule. Ils arrivent à la rive. Le sable est frais sous les bottes. Je fais le mur. Une poignée, puis une autre.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On met tes bottes. Victorina enfile ses bottes. Tu as fini tes bottes ? Oui, papa. On ferme la porte. Papa ferme la porte. Tu as ton sac, Victorina ? Oui, maman. Le chemin sent l'herbe mouillée, puis le fleuve. Le seau tape un peu, tout doux. Mon château va être grand. Oui, le sable t'attend. Ils arrivent à la rive. Le sable est encore un peu frais. Victorina pose le sac. Elle sort le seau. Le plastique n'est plus mouillé. Je fais le mur. Doucement, une poignée, puis une autre. Le sable fait un petit bruit. Un mur tout bas apparaît. Il tient, ce mur. Encore une poignée. Victorina appuie tout doucement. Le château a un petit coin rond.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On met tes bottes. Victorina enfile ses bottes. Tu as fini tes bottes ? Oui, papa. On ferme la porte. Papa ferme la porte. Tu as ton &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;, Victorina ? Oui, maman. Le chemin sent l'herbe, puis le fleuve. Le seau tape un peu contre sa hanche. Mon château va être grand ! Oui, le sable t'attend. Le sable luisant appelle, au bout du sentier. J'y vais avec le seau ! Elle pose le sac contre une racine. Elle part avec le seau seul. La poche vide manque sur sa hanche. Mon éclat ! Victorina s'arrête net. Elle refuse de foncer. Attends, je regarde. Le sac attend contre la racine. Dans la poche, l'éclat de caillou pèse. Tu le sens, dans le sac ? Oui. Elle revient, prend le sac. La sangle revient sur l'épaule. Ils arrivent à la rive. Le sable est frais sous les bottes. Je fais le mur. Une poignée, puis une autre.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Florence porte le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Papa ferme la porte. [pause]</t>
+          <t>On met tes bottes. Victorina enfile ses bottes. Tu as fini tes bottes ? Oui, papa. On ferme la porte. Papa ferme la porte. Tu as ton &lt;emphasis&gt;sac&lt;/emphasis&gt;, Victorina ? Oui, maman. Le chemin sent l'herbe, puis le fleuve. Le seau tape un peu contre sa hanche. Mon château va être grand ! Oui, le sable t'attend. Le sable luisant appelle, au bout du sentier. J'y vais avec le seau ! Elle pose le sac contre une racine. Elle part avec le seau seul. La poche vide manque sur sa hanche. Mon éclat ! Victorina s'arrête net. Elle refuse de foncer. Attends, je regarde. Le sac attend contre la racine. Dans la poche, l'éclat de caillou pèse. Tu le sens, dans le sac ? Oui. Elle revient, prend le sac. La sangle revient sur l'épaule. Ils arrivent à la rive. Le sable est frais sous les bottes. Je fais le mur. Une poignée, puis une autre. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1820,7 +1830,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1828,10 +1838,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1861,23 +1871,23 @@
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1886,10 +1896,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1900,34 +1910,49 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_sans_le_sac; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
           <t>papa|On met tes bottes.
 narrateur|Victorina enfile ses bottes.
 papa|Tu as fini tes bottes ?
 enfant-f|Oui, papa.
-papa|On ferme la porte.
+maman|On ferme la porte.
 narrateur|Papa ferme la porte.
 maman|Tu as ton sac, Victorina ?
 enfant-f|Oui, maman.
-narrateur|Le chemin sent l'herbe mouillée, puis le fleuve.
-narrateur|Le seau tape un peu, tout doux.
-enfant-f|Mon château va être grand.
+narrateur|Le chemin sent l'herbe, puis le fleuve.
+narrateur|Le seau tape un peu contre sa hanche.
+enfant-f|Mon château va être grand !
 maman|Oui, le sable t'attend.
+narrateur|Le sable luisant appelle, au bout du sentier.
+enfant-f|J'y vais avec le seau !
+narrateur|Elle pose le sac contre une racine.
+narrateur|Elle part avec le seau seul.
+narrateur|La poche vide manque sur sa hanche.
+enfant-f|Mon éclat !
+narrateur|Victorina s'arrête net.
+narrateur|Elle refuse de foncer.
+enfant-f|Attends, je regarde.
+narrateur|Le sac attend contre la racine.
+narrateur|Dans la poche, l'éclat de caillou pèse.
+papa|Tu le sens, dans le sac ?
+enfant-f|Oui.
+narrateur|Elle revient, prend le sac.
+narrateur|La sangle revient sur l'épaule.
 narrateur|Ils arrivent à la rive.
-narrateur|Le sable est encore un peu frais.
-narrateur|Victorina pose le sac.
-narrateur|Elle sort le seau.
-narrateur|Le plastique n'est plus mouillé.
+narrateur|Le sable est frais sous les bottes.
 enfant-f|Je fais le mur.
-papa|Doucement, une poignée, puis une autre.
-narrateur|Le sable fait un petit bruit.
-narrateur|Un mur tout bas apparaît.
-maman|Il tient, ce mur.
-enfant-f|Encore une poignée.
-narrateur|Victorina appuie tout doucement.
-narrateur|Le château a un petit coin rond.</t>
+papa|Une poignée, puis une autre.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>chemin,fleuve,racine</t>
         </is>
       </c>
     </row>
@@ -1954,17 +1979,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le petit mur tient encore. L'eau du fleuve cliquette tout près. Mon château est là. Oui, tu l'as fait. Le seau rouge repose dans le sable. Le robinet du jardin est loin, maintenant. Merci pour le seau, Victorina. Le coin rond du château reste frais sous le doigt.</t>
+          <t>Un mur rond apparaît, bas. Il tient, ce mur. Une poignée, pour la tour. Victorina appuie, sans se presser. Elle ouvre la poche du sac. L'éclat de caillou luit, pâle. Comme sur la table ! Elle le pose dans le mur frais. Oui, tu l'as fait. Mon château est là. Tu le vois, le petit éclat ? Oui, maman. Le seau rouge repose dans le sable. L'eau du fleuve clapote contre la rive. La table du jardin est loin. Sur le mur, l'éclat de caillou garde un bord humide.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le petit mur tient encore. L'eau du fleuve cliquette tout près. Mon château est là. Oui, tu l'as fait. Le seau rouge repose dans le sable. Le robinet du jardin est loin, maintenant. Merci pour le seau, Victorina. Le coin rond du château reste frais sous le doigt.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Un mur rond apparaît, bas. Il tient, ce mur. Une poignée, pour la tour. Victorina appuie, sans se presser. Elle ouvre la poche du sac. L'&lt;emphasis level="moderate"&gt;éclat de caillou&lt;/emphasis&gt; luit, pâle. Comme sur la table ! Elle le pose dans le mur frais. Oui, tu l'as fait. Mon château est là. Tu le vois, le petit éclat ? Oui, maman. Le seau rouge repose dans le sable. L'eau du fleuve clapote contre la rive. La table du jardin est loin. Sur le mur, l'éclat de caillou garde un bord humide.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Un mur rond apparaît, bas. Il tient, ce mur. Une poignée, pour la tour. Victorina appuie, sans se presser. Elle ouvre la poche du sac. L'&lt;emphasis&gt;éclat de caillou&lt;/emphasis&gt; luit, pâle. Comme sur la table ! Elle le pose dans le mur frais. Oui, tu l'as fait. Mon château est là. Tu le vois, le petit éclat ? Oui, maman. Le seau rouge repose dans le sable. L'eau du fleuve clapote contre la rive. La table du jardin est loin. Sur le mur, l'éclat de caillou garde un bord humide.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2011,18 +2036,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2031,12 +2056,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2045,17 +2070,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de caillou</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2064,11 +2093,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2077,31 +2106,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_dessin_est_la_fenetre_du_mur; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le petit mur tient encore.
-narrateur|L'eau du fleuve cliquette tout près.
+          <t>narrateur|Un mur rond apparaît, bas.
+maman|Il tient, ce mur.
+enfant-f|Une poignée, pour la tour.
+narrateur|Victorina appuie, sans se presser.
+narrateur|Elle ouvre la poche du sac.
+narrateur|L'éclat de caillou luit, pâle.
+enfant-f|Comme sur la table !
+narrateur|Elle le pose dans le mur frais.
+papa|Oui, tu l'as fait.
 enfant-f|Mon château est là.
-papa|Oui, tu l'as fait.
+maman|Tu le vois, le petit éclat ?
+enfant-f|Oui, maman.
 narrateur|Le seau rouge repose dans le sable.
-narrateur|Le robinet du jardin est loin, maintenant.
-maman|Merci pour le seau, Victorina.
-narrateur|Le coin rond du château reste frais sous le doigt.</t>
+narrateur|L'eau du fleuve clapote contre la rive.
+narrateur|La table du jardin est loin.
+narrateur|Sur le mur, l'éclat de caillou garde un bord humide.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>sable,eau,mur</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2214,6 +2260,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>